<commit_message>
Addeding new clases and lots of fixes
</commit_message>
<xml_diff>
--- a/resources/data-imports/Core Imports/game_classes.xlsx
+++ b/resources/data-imports/Core Imports/game_classes.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="43">
   <si>
     <t>id</t>
   </si>
@@ -141,6 +141,9 @@
   </si>
   <si>
     <t>Apothecary</t>
+  </si>
+  <si>
+    <t>Buccaneer</t>
   </si>
 </sst>
 </file>
@@ -480,7 +483,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:S17"/>
+  <dimension ref="A1:S18"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="3.428" bestFit="true" customWidth="true" style="0"/>
@@ -1141,6 +1144,53 @@
         <v>50</v>
       </c>
     </row>
+    <row r="18" spans="1:19">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>42</v>
+      </c>
+      <c r="C18" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" t="s">
+        <v>21</v>
+      </c>
+      <c r="E18">
+        <v>3</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <v>2</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>3</v>
+      </c>
+      <c r="K18">
+        <v>2</v>
+      </c>
+      <c r="L18">
+        <v>0.03</v>
+      </c>
+      <c r="M18">
+        <v>0.03</v>
+      </c>
+      <c r="N18">
+        <v>0.03</v>
+      </c>
+      <c r="O18">
+        <v>0.05</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>